<commit_message>
give opportunity to have multiple identityreliability 408caca771a5f026de32e3deb45060601ebdd49e
</commit_message>
<xml_diff>
--- a/ig/nr-update-patient-ins/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/ig/nr-update-patient-ins/StructureDefinition-fr-core-patient-ins.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-26T11:00:29+00:00</t>
+    <t>2024-02-26T11:04:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -5160,7 +5160,7 @@
         <v>89</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H20" t="s" s="2">
         <v>81</v>

</xml_diff>